<commit_message>
tp & charm price
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
+++ b/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B381167E-7B51-404B-9EAA-241D571E6CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F4FB0A4-4901-400C-A33F-61403E0338E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1088,7 +1088,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1103,6 +1103,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="42"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1139,12 +1145,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3277,269 +3286,269 @@
       </c>
       <c r="AC20" s="2"/>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:29" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B21" s="3">
-        <v>1</v>
-      </c>
-      <c r="C21" s="3" t="s">
+      <c r="B21" s="5">
+        <v>1</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="5">
         <v>2</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="6">
         <v>780</v>
       </c>
-      <c r="G21" s="2">
+      <c r="G21" s="6">
         <v>300</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="H21" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="I21" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J21" s="3" t="s">
+      <c r="J21" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="K21" s="3">
-        <v>0</v>
-      </c>
-      <c r="L21" s="3">
-        <v>1</v>
-      </c>
-      <c r="M21" s="3">
-        <v>0</v>
-      </c>
-      <c r="N21" s="3">
-        <v>0</v>
-      </c>
-      <c r="O21" s="3">
-        <v>0</v>
-      </c>
-      <c r="P21" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="3">
-        <v>0</v>
-      </c>
-      <c r="R21" s="3">
+      <c r="K21" s="5">
+        <v>0</v>
+      </c>
+      <c r="L21" s="5">
+        <v>15909</v>
+      </c>
+      <c r="M21" s="5">
+        <v>0</v>
+      </c>
+      <c r="N21" s="5">
+        <v>0</v>
+      </c>
+      <c r="O21" s="5">
+        <v>0</v>
+      </c>
+      <c r="P21" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="5">
+        <v>0</v>
+      </c>
+      <c r="R21" s="5">
         <v>35</v>
       </c>
-      <c r="S21" s="3">
+      <c r="S21" s="5">
         <v>-1</v>
       </c>
-      <c r="T21" s="3">
-        <v>1</v>
-      </c>
-      <c r="U21" s="3">
-        <v>0</v>
-      </c>
-      <c r="V21" s="3">
-        <v>0</v>
-      </c>
-      <c r="W21" s="3">
-        <v>1</v>
-      </c>
-      <c r="X21" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y21" s="2" t="str">
+      <c r="T21" s="5">
+        <v>1</v>
+      </c>
+      <c r="U21" s="5">
+        <v>0</v>
+      </c>
+      <c r="V21" s="5">
+        <v>0</v>
+      </c>
+      <c r="W21" s="5">
+        <v>1</v>
+      </c>
+      <c r="X21" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y21" s="6" t="str">
         <f t="shared" si="0"/>
         <v>tiqcsa01</v>
       </c>
-      <c r="Z21" s="3">
-        <v>1</v>
-      </c>
-      <c r="AA21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC21" s="2"/>
-    </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="Z21" s="5">
+        <v>1</v>
+      </c>
+      <c r="AA21" s="5">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="5">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="6"/>
+    </row>
+    <row r="22" spans="1:29" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B22" s="3">
-        <v>1</v>
-      </c>
-      <c r="C22" s="3" t="s">
+      <c r="B22" s="5">
+        <v>1</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="5">
         <v>2</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="6">
         <v>780</v>
       </c>
-      <c r="G22" s="2">
+      <c r="G22" s="6">
         <v>300</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="H22" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="I22" s="3" t="s">
+      <c r="I22" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J22" s="3" t="s">
+      <c r="J22" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="K22" s="3">
-        <v>0</v>
-      </c>
-      <c r="L22" s="3">
-        <v>1</v>
-      </c>
-      <c r="M22" s="3">
-        <v>0</v>
-      </c>
-      <c r="N22" s="3">
-        <v>0</v>
-      </c>
-      <c r="O22" s="3">
-        <v>0</v>
-      </c>
-      <c r="P22" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="3">
-        <v>0</v>
-      </c>
-      <c r="R22" s="3">
+      <c r="K22" s="5">
+        <v>0</v>
+      </c>
+      <c r="L22" s="5">
+        <v>15909</v>
+      </c>
+      <c r="M22" s="5">
+        <v>0</v>
+      </c>
+      <c r="N22" s="5">
+        <v>0</v>
+      </c>
+      <c r="O22" s="5">
+        <v>0</v>
+      </c>
+      <c r="P22" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="5">
+        <v>0</v>
+      </c>
+      <c r="R22" s="5">
         <v>35</v>
       </c>
-      <c r="S22" s="3">
+      <c r="S22" s="5">
         <v>-1</v>
       </c>
-      <c r="T22" s="3">
-        <v>1</v>
-      </c>
-      <c r="U22" s="3">
-        <v>0</v>
-      </c>
-      <c r="V22" s="3">
-        <v>0</v>
-      </c>
-      <c r="W22" s="3">
-        <v>1</v>
-      </c>
-      <c r="X22" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y22" s="2" t="str">
+      <c r="T22" s="5">
+        <v>1</v>
+      </c>
+      <c r="U22" s="5">
+        <v>0</v>
+      </c>
+      <c r="V22" s="5">
+        <v>0</v>
+      </c>
+      <c r="W22" s="5">
+        <v>1</v>
+      </c>
+      <c r="X22" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y22" s="6" t="str">
         <f t="shared" si="0"/>
         <v>tiqcsa02</v>
       </c>
-      <c r="Z22" s="3">
-        <v>1</v>
-      </c>
-      <c r="AA22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC22" s="2"/>
-    </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="Z22" s="5">
+        <v>1</v>
+      </c>
+      <c r="AA22" s="5">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="5">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="6"/>
+    </row>
+    <row r="23" spans="1:29" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B23" s="3">
-        <v>1</v>
-      </c>
-      <c r="C23" s="3" t="s">
+      <c r="B23" s="5">
+        <v>1</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="5">
         <v>2</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="6">
         <v>780</v>
       </c>
-      <c r="G23" s="2">
+      <c r="G23" s="6">
         <v>300</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H23" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="I23" s="3" t="s">
+      <c r="I23" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J23" s="3" t="s">
+      <c r="J23" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="K23" s="3">
-        <v>0</v>
-      </c>
-      <c r="L23" s="3">
-        <v>1</v>
-      </c>
-      <c r="M23" s="3">
-        <v>0</v>
-      </c>
-      <c r="N23" s="3">
-        <v>0</v>
-      </c>
-      <c r="O23" s="3">
-        <v>0</v>
-      </c>
-      <c r="P23" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="3">
-        <v>0</v>
-      </c>
-      <c r="R23" s="3">
+      <c r="K23" s="5">
+        <v>0</v>
+      </c>
+      <c r="L23" s="5">
+        <v>15909</v>
+      </c>
+      <c r="M23" s="5">
+        <v>0</v>
+      </c>
+      <c r="N23" s="5">
+        <v>0</v>
+      </c>
+      <c r="O23" s="5">
+        <v>0</v>
+      </c>
+      <c r="P23" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="5">
+        <v>0</v>
+      </c>
+      <c r="R23" s="5">
         <v>35</v>
       </c>
-      <c r="S23" s="3">
+      <c r="S23" s="5">
         <v>-1</v>
       </c>
-      <c r="T23" s="3">
-        <v>1</v>
-      </c>
-      <c r="U23" s="3">
-        <v>0</v>
-      </c>
-      <c r="V23" s="3">
-        <v>0</v>
-      </c>
-      <c r="W23" s="3">
-        <v>1</v>
-      </c>
-      <c r="X23" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y23" s="2" t="str">
+      <c r="T23" s="5">
+        <v>1</v>
+      </c>
+      <c r="U23" s="5">
+        <v>0</v>
+      </c>
+      <c r="V23" s="5">
+        <v>0</v>
+      </c>
+      <c r="W23" s="5">
+        <v>1</v>
+      </c>
+      <c r="X23" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y23" s="6" t="str">
         <f t="shared" si="0"/>
         <v>tiqcsa03</v>
       </c>
-      <c r="Z23" s="3">
-        <v>1</v>
-      </c>
-      <c r="AA23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC23" s="2"/>
+      <c r="Z23" s="5">
+        <v>1</v>
+      </c>
+      <c r="AA23" s="5">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="5">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="6"/>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
@@ -11680,7 +11689,7 @@
       </c>
       <c r="I21">
         <f>TOWNItem!L21</f>
-        <v>1</v>
+        <v>15909</v>
       </c>
       <c r="J21">
         <f>TOWNItem!M21</f>
@@ -11790,7 +11799,7 @@
       </c>
       <c r="I22">
         <f>TOWNItem!L22</f>
-        <v>1</v>
+        <v>15909</v>
       </c>
       <c r="J22">
         <f>TOWNItem!M22</f>
@@ -11900,7 +11909,7 @@
       </c>
       <c r="I23">
         <f>TOWNItem!L23</f>
-        <v>1</v>
+        <v>15909</v>
       </c>
       <c r="J23">
         <f>TOWNItem!M23</f>

</xml_diff>

<commit_message>
ps hq tp fix
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
+++ b/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F4FB0A4-4901-400C-A33F-61403E0338E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA14E0F7-C3AC-4570-A8BB-3EAF1B460126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8302,269 +8302,269 @@
       </c>
       <c r="AC77" s="2"/>
     </row>
-    <row r="78" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A78" s="3" t="s">
+    <row r="78" spans="1:29" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="B78" s="3">
-        <v>1</v>
-      </c>
-      <c r="C78" s="3" t="s">
+      <c r="B78" s="5">
+        <v>1</v>
+      </c>
+      <c r="C78" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D78" s="3">
+      <c r="D78" s="5">
         <v>59</v>
       </c>
-      <c r="E78" s="3" t="s">
+      <c r="E78" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="F78" s="2">
+      <c r="F78" s="6">
         <v>780</v>
       </c>
-      <c r="G78" s="2">
+      <c r="G78" s="6">
         <v>300</v>
       </c>
-      <c r="H78" s="3" t="s">
+      <c r="H78" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="I78" s="3" t="s">
+      <c r="I78" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="J78" s="3" t="s">
+      <c r="J78" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="K78" s="3">
-        <v>0</v>
-      </c>
-      <c r="L78" s="3">
-        <v>1</v>
-      </c>
-      <c r="M78" s="3">
-        <v>0</v>
-      </c>
-      <c r="N78" s="3">
-        <v>0</v>
-      </c>
-      <c r="O78" s="3">
-        <v>0</v>
-      </c>
-      <c r="P78" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q78" s="3">
-        <v>0</v>
-      </c>
-      <c r="R78" s="3">
-        <v>1</v>
-      </c>
-      <c r="S78" s="3">
+      <c r="K78" s="5">
+        <v>0</v>
+      </c>
+      <c r="L78" s="5">
+        <v>1818182</v>
+      </c>
+      <c r="M78" s="5">
+        <v>0</v>
+      </c>
+      <c r="N78" s="5">
+        <v>0</v>
+      </c>
+      <c r="O78" s="5">
+        <v>0</v>
+      </c>
+      <c r="P78" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="5">
+        <v>0</v>
+      </c>
+      <c r="R78" s="5">
+        <v>1</v>
+      </c>
+      <c r="S78" s="5">
         <v>-1</v>
       </c>
-      <c r="T78" s="3">
-        <v>1</v>
-      </c>
-      <c r="U78" s="3">
-        <v>0</v>
-      </c>
-      <c r="V78" s="3">
-        <v>0</v>
-      </c>
-      <c r="W78" s="3">
-        <v>1</v>
-      </c>
-      <c r="X78" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y78" s="2" t="str">
+      <c r="T78" s="5">
+        <v>1</v>
+      </c>
+      <c r="U78" s="5">
+        <v>0</v>
+      </c>
+      <c r="V78" s="5">
+        <v>0</v>
+      </c>
+      <c r="W78" s="5">
+        <v>0</v>
+      </c>
+      <c r="X78" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y78" s="6" t="str">
         <f t="shared" si="1"/>
         <v>tiqbpc01</v>
       </c>
-      <c r="Z78" s="3">
-        <v>1</v>
-      </c>
-      <c r="AA78" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB78" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC78" s="2"/>
-    </row>
-    <row r="79" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A79" s="3" t="s">
+      <c r="Z78" s="5">
+        <v>1</v>
+      </c>
+      <c r="AA78" s="5">
+        <v>0</v>
+      </c>
+      <c r="AB78" s="5">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="6"/>
+    </row>
+    <row r="79" spans="1:29" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="B79" s="3">
-        <v>1</v>
-      </c>
-      <c r="C79" s="3" t="s">
+      <c r="B79" s="5">
+        <v>1</v>
+      </c>
+      <c r="C79" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D79" s="3">
+      <c r="D79" s="5">
         <v>59</v>
       </c>
-      <c r="E79" s="3" t="s">
+      <c r="E79" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="F79" s="2">
+      <c r="F79" s="6">
         <v>780</v>
       </c>
-      <c r="G79" s="2">
+      <c r="G79" s="6">
         <v>300</v>
       </c>
-      <c r="H79" s="3" t="s">
+      <c r="H79" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="I79" s="3" t="s">
+      <c r="I79" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="J79" s="3" t="s">
+      <c r="J79" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="K79" s="3">
-        <v>0</v>
-      </c>
-      <c r="L79" s="3">
-        <v>1</v>
-      </c>
-      <c r="M79" s="3">
-        <v>0</v>
-      </c>
-      <c r="N79" s="3">
-        <v>0</v>
-      </c>
-      <c r="O79" s="3">
-        <v>0</v>
-      </c>
-      <c r="P79" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q79" s="3">
-        <v>0</v>
-      </c>
-      <c r="R79" s="3">
-        <v>1</v>
-      </c>
-      <c r="S79" s="3">
+      <c r="K79" s="5">
+        <v>0</v>
+      </c>
+      <c r="L79" s="5">
+        <v>1818182</v>
+      </c>
+      <c r="M79" s="5">
+        <v>0</v>
+      </c>
+      <c r="N79" s="5">
+        <v>0</v>
+      </c>
+      <c r="O79" s="5">
+        <v>0</v>
+      </c>
+      <c r="P79" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="5">
+        <v>0</v>
+      </c>
+      <c r="R79" s="5">
+        <v>1</v>
+      </c>
+      <c r="S79" s="5">
         <v>-1</v>
       </c>
-      <c r="T79" s="3">
-        <v>1</v>
-      </c>
-      <c r="U79" s="3">
-        <v>0</v>
-      </c>
-      <c r="V79" s="3">
-        <v>0</v>
-      </c>
-      <c r="W79" s="3">
-        <v>1</v>
-      </c>
-      <c r="X79" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y79" s="2" t="str">
+      <c r="T79" s="5">
+        <v>1</v>
+      </c>
+      <c r="U79" s="5">
+        <v>0</v>
+      </c>
+      <c r="V79" s="5">
+        <v>0</v>
+      </c>
+      <c r="W79" s="5">
+        <v>0</v>
+      </c>
+      <c r="X79" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y79" s="6" t="str">
         <f t="shared" si="1"/>
         <v>tiqcpc01</v>
       </c>
-      <c r="Z79" s="3">
-        <v>1</v>
-      </c>
-      <c r="AA79" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB79" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC79" s="2"/>
-    </row>
-    <row r="80" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A80" s="3" t="s">
+      <c r="Z79" s="5">
+        <v>1</v>
+      </c>
+      <c r="AA79" s="5">
+        <v>0</v>
+      </c>
+      <c r="AB79" s="5">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="6"/>
+    </row>
+    <row r="80" spans="1:29" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B80" s="3">
-        <v>1</v>
-      </c>
-      <c r="C80" s="3" t="s">
+      <c r="B80" s="5">
+        <v>1</v>
+      </c>
+      <c r="C80" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D80" s="3">
+      <c r="D80" s="5">
         <v>59</v>
       </c>
-      <c r="E80" s="3" t="s">
+      <c r="E80" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="F80" s="2">
+      <c r="F80" s="6">
         <v>780</v>
       </c>
-      <c r="G80" s="2">
+      <c r="G80" s="6">
         <v>300</v>
       </c>
-      <c r="H80" s="3" t="s">
+      <c r="H80" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="I80" s="3" t="s">
+      <c r="I80" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="J80" s="3" t="s">
+      <c r="J80" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="K80" s="3">
-        <v>0</v>
-      </c>
-      <c r="L80" s="3">
-        <v>1</v>
-      </c>
-      <c r="M80" s="3">
-        <v>0</v>
-      </c>
-      <c r="N80" s="3">
-        <v>0</v>
-      </c>
-      <c r="O80" s="3">
-        <v>0</v>
-      </c>
-      <c r="P80" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q80" s="3">
-        <v>0</v>
-      </c>
-      <c r="R80" s="3">
-        <v>1</v>
-      </c>
-      <c r="S80" s="3">
+      <c r="K80" s="5">
+        <v>0</v>
+      </c>
+      <c r="L80" s="5">
+        <v>1818182</v>
+      </c>
+      <c r="M80" s="5">
+        <v>0</v>
+      </c>
+      <c r="N80" s="5">
+        <v>0</v>
+      </c>
+      <c r="O80" s="5">
+        <v>0</v>
+      </c>
+      <c r="P80" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="5">
+        <v>0</v>
+      </c>
+      <c r="R80" s="5">
+        <v>1</v>
+      </c>
+      <c r="S80" s="5">
         <v>-1</v>
       </c>
-      <c r="T80" s="3">
-        <v>1</v>
-      </c>
-      <c r="U80" s="3">
-        <v>0</v>
-      </c>
-      <c r="V80" s="3">
-        <v>0</v>
-      </c>
-      <c r="W80" s="3">
-        <v>1</v>
-      </c>
-      <c r="X80" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y80" s="2" t="str">
+      <c r="T80" s="5">
+        <v>1</v>
+      </c>
+      <c r="U80" s="5">
+        <v>0</v>
+      </c>
+      <c r="V80" s="5">
+        <v>0</v>
+      </c>
+      <c r="W80" s="5">
+        <v>0</v>
+      </c>
+      <c r="X80" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y80" s="6" t="str">
         <f t="shared" si="1"/>
         <v>tiqapc01</v>
       </c>
-      <c r="Z80" s="3">
-        <v>1</v>
-      </c>
-      <c r="AA80" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB80" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC80" s="2"/>
+      <c r="Z80" s="5">
+        <v>1</v>
+      </c>
+      <c r="AA80" s="5">
+        <v>0</v>
+      </c>
+      <c r="AB80" s="5">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="6"/>
     </row>
     <row r="81" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
@@ -17959,7 +17959,7 @@
       </c>
       <c r="I78">
         <f>TOWNItem!L78</f>
-        <v>1</v>
+        <v>1818182</v>
       </c>
       <c r="J78">
         <f>TOWNItem!M78</f>
@@ -17995,7 +17995,7 @@
       </c>
       <c r="R78">
         <f>TOWNItem!W78</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S78" s="4">
         <v>75</v>
@@ -18069,7 +18069,7 @@
       </c>
       <c r="I79">
         <f>TOWNItem!L79</f>
-        <v>1</v>
+        <v>1818182</v>
       </c>
       <c r="J79">
         <f>TOWNItem!M79</f>
@@ -18105,7 +18105,7 @@
       </c>
       <c r="R79">
         <f>TOWNItem!W79</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S79" s="4">
         <v>76</v>
@@ -18179,7 +18179,7 @@
       </c>
       <c r="I80">
         <f>TOWNItem!L80</f>
-        <v>1</v>
+        <v>1818182</v>
       </c>
       <c r="J80">
         <f>TOWNItem!M80</f>
@@ -18215,7 +18215,7 @@
       </c>
       <c r="R80">
         <f>TOWNItem!W80</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S80" s="4">
         <v>77</v>

</xml_diff>

<commit_message>
cbt fix starting fix
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
+++ b/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA14E0F7-C3AC-4570-A8BB-3EAF1B460126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6583F318-0B34-41AF-8A0C-C4B0838EBB21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TOWNItem" sheetId="1" r:id="rId1"/>
@@ -1172,9 +1172,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1212,9 +1212,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1247,26 +1247,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1299,26 +1282,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8361,7 +8327,7 @@
         <v>-1</v>
       </c>
       <c r="T78" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U78" s="5">
         <v>0</v>
@@ -8449,7 +8415,7 @@
         <v>-1</v>
       </c>
       <c r="T79" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U79" s="5">
         <v>0</v>
@@ -8537,7 +8503,7 @@
         <v>-1</v>
       </c>
       <c r="T80" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U80" s="5">
         <v>0</v>
@@ -17987,7 +17953,7 @@
       </c>
       <c r="P78">
         <f>TOWNItem!T78</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q78">
         <f>TOWNItem!V78</f>
@@ -18097,7 +18063,7 @@
       </c>
       <c r="P79">
         <f>TOWNItem!T79</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q79">
         <f>TOWNItem!V79</f>
@@ -18207,7 +18173,7 @@
       </c>
       <c r="P80">
         <f>TOWNItem!T80</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q80">
         <f>TOWNItem!V80</f>

</xml_diff>

<commit_message>
elan tp & scanner price
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
+++ b/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31740349-C228-403C-9D04-6F8A30A7B76F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FEE81D8-4AB9-459C-AF52-F365CA01A056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TOWNItem" sheetId="1" r:id="rId1"/>
@@ -1172,9 +1172,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1212,9 +1212,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1247,9 +1247,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1282,9 +1299,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3076,93 +3110,93 @@
       </c>
       <c r="AC18" s="2"/>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:29" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="3">
-        <v>1</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B19" s="5">
+        <v>1</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D19" s="3">
-        <v>1</v>
-      </c>
-      <c r="E19" s="3" t="s">
+      <c r="D19" s="5">
+        <v>1</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="6">
         <v>780</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="6">
         <v>300</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="H19" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="I19" s="3" t="s">
+      <c r="I19" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="J19" s="3" t="s">
+      <c r="J19" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="K19" s="3">
-        <v>0</v>
-      </c>
-      <c r="L19" s="3">
-        <v>1000</v>
-      </c>
-      <c r="M19" s="3">
-        <v>0</v>
-      </c>
-      <c r="N19" s="3">
-        <v>0</v>
-      </c>
-      <c r="O19" s="3">
-        <v>0</v>
-      </c>
-      <c r="P19" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="3">
+      <c r="K19" s="5">
+        <v>0</v>
+      </c>
+      <c r="L19" s="5">
+        <v>455</v>
+      </c>
+      <c r="M19" s="5">
+        <v>0</v>
+      </c>
+      <c r="N19" s="5">
+        <v>0</v>
+      </c>
+      <c r="O19" s="5">
+        <v>0</v>
+      </c>
+      <c r="P19" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="5">
         <v>50</v>
       </c>
-      <c r="R19" s="3">
+      <c r="R19" s="5">
         <v>45</v>
       </c>
-      <c r="S19" s="3">
+      <c r="S19" s="5">
         <v>-1</v>
       </c>
-      <c r="T19" s="3">
-        <v>1</v>
-      </c>
-      <c r="U19" s="3">
-        <v>1</v>
-      </c>
-      <c r="V19" s="3">
-        <v>1</v>
-      </c>
-      <c r="W19" s="3">
-        <v>1</v>
-      </c>
-      <c r="X19" s="2">
-        <v>1</v>
-      </c>
-      <c r="Y19" s="2" t="str">
+      <c r="T19" s="5">
+        <v>1</v>
+      </c>
+      <c r="U19" s="5">
+        <v>1</v>
+      </c>
+      <c r="V19" s="5">
+        <v>1</v>
+      </c>
+      <c r="W19" s="5">
+        <v>1</v>
+      </c>
+      <c r="X19" s="6">
+        <v>1</v>
+      </c>
+      <c r="Y19" s="6" t="str">
         <f t="shared" si="0"/>
         <v>tiqell01</v>
       </c>
-      <c r="Z19" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC19" s="2"/>
+      <c r="Z19" s="5">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="5">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="5">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="6"/>
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
@@ -11435,7 +11469,7 @@
       </c>
       <c r="I19">
         <f>TOWNItem!L19</f>
-        <v>1000</v>
+        <v>455</v>
       </c>
       <c r="J19">
         <f>TOWNItem!M19</f>

</xml_diff>

<commit_message>
Premium HQ TP price to 1m
</commit_message>
<xml_diff>
--- a/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
+++ b/gu_in/Item.edf/22_TownItem/TOWNItem.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FEE81D8-4AB9-459C-AF52-F365CA01A056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2456C88-C0D6-4265-AFEF-A143A7FBB9AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="945" yWindow="1050" windowWidth="17565" windowHeight="11205" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TOWNItem" sheetId="1" r:id="rId1"/>
@@ -8337,7 +8337,7 @@
         <v>0</v>
       </c>
       <c r="L78" s="5">
-        <v>1818182</v>
+        <v>909091</v>
       </c>
       <c r="M78" s="5">
         <v>0</v>
@@ -8425,7 +8425,7 @@
         <v>0</v>
       </c>
       <c r="L79" s="5">
-        <v>1818182</v>
+        <v>909091</v>
       </c>
       <c r="M79" s="5">
         <v>0</v>
@@ -8513,7 +8513,7 @@
         <v>0</v>
       </c>
       <c r="L80" s="5">
-        <v>1818182</v>
+        <v>909091</v>
       </c>
       <c r="M80" s="5">
         <v>0</v>
@@ -17959,7 +17959,7 @@
       </c>
       <c r="I78">
         <f>TOWNItem!L78</f>
-        <v>1818182</v>
+        <v>909091</v>
       </c>
       <c r="J78">
         <f>TOWNItem!M78</f>
@@ -18069,7 +18069,7 @@
       </c>
       <c r="I79">
         <f>TOWNItem!L79</f>
-        <v>1818182</v>
+        <v>909091</v>
       </c>
       <c r="J79">
         <f>TOWNItem!M79</f>
@@ -18179,7 +18179,7 @@
       </c>
       <c r="I80">
         <f>TOWNItem!L80</f>
-        <v>1818182</v>
+        <v>909091</v>
       </c>
       <c r="J80">
         <f>TOWNItem!M80</f>

</xml_diff>